<commit_message>
Completar Parte 1: hoja 'Gastos captura' (tabla dual manual/XML + conceptos dinámicos) + entrega
- Concentrado_CFDI_AUTOMATIZADO.xlsx: agrega hoja 'Gastos captura' con Tabla de Excel
  (Mes/Categoria/Concepto/Importe/Origen), validaciones, resumen por categoria con % y
  meta 50/20/30, y gráfica de pastel. Inyectada vía XML conservando todo lo existente.
- Tutorial actualizado con la nueva hoja.
- ENTREGA_Parte1.md: documento de entrega que resume todo lo cotizado.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016pudwoamudm6kkBbcBjEzD
</commit_message>
<xml_diff>
--- a/Concentrado_CFDI_AUTOMATIZADO.xlsx
+++ b/Concentrado_CFDI_AUTOMATIZADO.xlsx
@@ -22,6 +22,7 @@
     <sheet name="detalle" sheetId="31" r:id="rId6"/>
     <sheet name="concentrado" sheetId="32" r:id="rId7"/>
     <sheet name="tabulador" sheetId="4" r:id="rId8"/>
+    <sheet name="Gastos captura" sheetId="34" r:id="rId21"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">fabi!$A$1:$DH$5</definedName>
@@ -5202,6 +5203,58 @@
           <val>
             <numRef>
               <f>'DASHBOARD'!$K$7:$K$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Gastos por categoria (mes elegido)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Gastos captura'!$H$6:$H$8</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Gastos captura'!$I$6:$I$8</f>
             </numRef>
           </val>
         </ser>
@@ -6729,6 +6782,33 @@
 </wsDr>
 </file>
 
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3600000" cy="2340000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="angel murillo" refreshedDate="45374.702363078701" createdVersion="5" refreshedVersion="5" minRefreshableVersion="3" recordCount="24" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
   <cacheSource type="worksheet">
@@ -7711,6 +7791,20 @@
 </table>
 </file>
 
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Gastos" displayName="Gastos" ref="A4:E28" headerRowCount="1">
+  <autoFilter ref="A4:E28"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Mes"/>
+    <tableColumn id="2" name="Categoria"/>
+    <tableColumn id="3" name="Concepto"/>
+    <tableColumn id="4" name="Importe"/>
+    <tableColumn id="5" name="Origen"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
@@ -9185,6 +9279,662 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Gastos — Captura (manual o XML)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Agrega los renglones/conceptos que necesites. Marca el Mes (1-12), la Categoria (Basico/Lujo/Ahorro), el Importe y el Origen.</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Resumen por categoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Mes:</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Categoria</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Importe</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Origen</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Basico</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Renta / Hipoteca</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Categoria</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Monto</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>% real</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Basico</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Agua (CESPT)</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Basico</t>
+        </is>
+      </c>
+      <c r="I6" s="9">
+        <f>SUMIFS(Gastos[Importe],Gastos[Categoria],"Basico",Gastos[Mes],$I$3)</f>
+        <v/>
+      </c>
+      <c r="J6" s="10">
+        <f>IFERROR(I6/$I$9,0)</f>
+        <v/>
+      </c>
+      <c r="K6" s="11" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Basico</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Luz (CFE)</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Lujo</t>
+        </is>
+      </c>
+      <c r="I7" s="9">
+        <f>SUMIFS(Gastos[Importe],Gastos[Categoria],"Lujo",Gastos[Mes],$I$3)</f>
+        <v/>
+      </c>
+      <c r="J7" s="10">
+        <f>IFERROR(I7/$I$9,0)</f>
+        <v/>
+      </c>
+      <c r="K7" s="11" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Basico</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>Ahorro</t>
+        </is>
+      </c>
+      <c r="I8" s="9">
+        <f>SUMIFS(Gastos[Importe],Gastos[Categoria],"Ahorro",Gastos[Mes],$I$3)</f>
+        <v/>
+      </c>
+      <c r="J8" s="10">
+        <f>IFERROR(I8/$I$9,0)</f>
+        <v/>
+      </c>
+      <c r="K8" s="11" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Basico</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="I9" s="13">
+        <f>SUM(I6:I8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Basico</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Telefono / Recargas</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Basico</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Mantenimiento privada</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Basico</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Predial</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Basico</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Despensa / Supermercado</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Basico</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Mercado</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Basico</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Transporte / Pasajes</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Basico</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Salud / Medicamentos</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Basico</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Escuela / Colegiaturas</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Lujo</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Restaurantes / Comidas</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Lujo</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Cine / Entretenimiento</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Lujo</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Ropa / Cosmeticos</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Lujo</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Libros / Cafe / Golosinas</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Lujo</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Mascotas / Veterinario</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Lujo</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Viajes / Hotel</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Lujo</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Cumpleanos / Regalos</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Ahorro</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Tarjeta de credito</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Ahorro</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Prestamo personal</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Ahorro</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Pago a capital / Empenos</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Ahorro</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Ahorro / Fondo emergencia</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="4">
+    <dataValidation sqref="B5:B28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Basico,Lujo,Ahorro"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E5:E28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Manual,XML"</formula1>
+    </dataValidation>
+    <dataValidation sqref="A5:A28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1,2,3,4,5,6,7,8,9,10,11,12"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1,2,3,4,5,6,7,8,9,10,11,12"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>

</xml_diff>

<commit_message>
Fix aviso de reparación de Excel: metadatos app.xml (10 hojas), quitar <v> vacíos, RFC por nombre definido, y relación calcChain colgante en CORREGIDO
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016pudwoamudm6kkBbcBjEzD
</commit_message>
<xml_diff>
--- a/Concentrado_CFDI_AUTOMATIZADO.xlsx
+++ b/Concentrado_CFDI_AUTOMATIZADO.xlsx
@@ -25,6 +25,7 @@
     <sheet name="Gastos captura" sheetId="34" r:id="rId21"/>
   </sheets>
   <definedNames>
+    <definedName name="RFCList">fabi!$F$2:$F$1000</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">fabi!$A$1:$DH$5</definedName>
     <definedName name="entradas">Tabla9[]</definedName>
     <definedName name="gastos">'hoja de gastos'!$A$2:$E$98</definedName>
@@ -9421,11 +9422,9 @@
       </c>
       <c r="I6" s="9">
         <f>SUMIFS(Gastos[Importe],Gastos[Categoria],"Basico",Gastos[Mes],$I$3)</f>
-        <v/>
       </c>
       <c r="J6" s="10">
         <f>IFERROR(I6/$I$9,0)</f>
-        <v/>
       </c>
       <c r="K6" s="11" t="n">
         <v>0.5</v>
@@ -9457,11 +9456,9 @@
       </c>
       <c r="I7" s="9">
         <f>SUMIFS(Gastos[Importe],Gastos[Categoria],"Lujo",Gastos[Mes],$I$3)</f>
-        <v/>
       </c>
       <c r="J7" s="10">
         <f>IFERROR(I7/$I$9,0)</f>
-        <v/>
       </c>
       <c r="K7" s="11" t="n">
         <v>0.2</v>
@@ -9493,11 +9490,9 @@
       </c>
       <c r="I8" s="9">
         <f>SUMIFS(Gastos[Importe],Gastos[Categoria],"Ahorro",Gastos[Mes],$I$3)</f>
-        <v/>
       </c>
       <c r="J8" s="10">
         <f>IFERROR(I8/$I$9,0)</f>
-        <v/>
       </c>
       <c r="K8" s="11" t="n">
         <v>0.3</v>
@@ -9529,7 +9524,6 @@
       </c>
       <c r="I9" s="13">
         <f>SUM(I6:I8)</f>
-        <v/>
       </c>
     </row>
     <row r="10">
@@ -15733,29 +15727,23 @@
       </c>
       <c r="K7">
         <f>INDEX($B$12:$B$23,$C$5)</f>
-        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6">
         <f>INDEX($B$12:$B$23,$C$5)</f>
-        <v/>
       </c>
       <c r="B8" s="6">
         <f>INDEX($C$12:$C$23,$C$5)</f>
-        <v/>
       </c>
       <c r="C8" s="6">
         <f>INDEX($D$12:$D$23,$C$5)</f>
-        <v/>
       </c>
       <c r="D8" s="7">
         <f>INDEX($E$12:$E$23,$C$5)</f>
-        <v/>
       </c>
       <c r="E8" s="7">
         <f>INDEX($F$12:$F$23,$C$5)</f>
-        <v/>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -15764,7 +15752,6 @@
       </c>
       <c r="K8">
         <f>INDEX($C$12:$C$23,$C$5)</f>
-        <v/>
       </c>
     </row>
     <row r="11">
@@ -15812,23 +15799,18 @@
       </c>
       <c r="B12" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H12,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$BF$2:$BF$1000)</f>
-        <v/>
       </c>
       <c r="C12" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H12,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CA$2:$CA$1000)</f>
-        <v/>
       </c>
       <c r="D12" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H12,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CD$2:$CD$1000)</f>
-        <v/>
       </c>
       <c r="E12" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H12,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0))</f>
-        <v/>
       </c>
       <c r="F12" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H12,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*(--(fabi!$J$2:$J$1000&lt;&gt;"VIGENTE")))</f>
-        <v/>
       </c>
       <c r="H12" t="n">
         <v>1</v>
@@ -15842,23 +15824,18 @@
       </c>
       <c r="B13" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H13,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$BF$2:$BF$1000)</f>
-        <v/>
       </c>
       <c r="C13" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H13,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CA$2:$CA$1000)</f>
-        <v/>
       </c>
       <c r="D13" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H13,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CD$2:$CD$1000)</f>
-        <v/>
       </c>
       <c r="E13" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H13,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0))</f>
-        <v/>
       </c>
       <c r="F13" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H13,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*(--(fabi!$J$2:$J$1000&lt;&gt;"VIGENTE")))</f>
-        <v/>
       </c>
       <c r="H13" t="n">
         <v>2</v>
@@ -15872,23 +15849,18 @@
       </c>
       <c r="B14" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H14,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$BF$2:$BF$1000)</f>
-        <v/>
       </c>
       <c r="C14" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H14,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CA$2:$CA$1000)</f>
-        <v/>
       </c>
       <c r="D14" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H14,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CD$2:$CD$1000)</f>
-        <v/>
       </c>
       <c r="E14" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H14,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0))</f>
-        <v/>
       </c>
       <c r="F14" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H14,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*(--(fabi!$J$2:$J$1000&lt;&gt;"VIGENTE")))</f>
-        <v/>
       </c>
       <c r="H14" t="n">
         <v>3</v>
@@ -15902,23 +15874,18 @@
       </c>
       <c r="B15" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H15,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$BF$2:$BF$1000)</f>
-        <v/>
       </c>
       <c r="C15" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H15,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CA$2:$CA$1000)</f>
-        <v/>
       </c>
       <c r="D15" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H15,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CD$2:$CD$1000)</f>
-        <v/>
       </c>
       <c r="E15" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H15,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0))</f>
-        <v/>
       </c>
       <c r="F15" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H15,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*(--(fabi!$J$2:$J$1000&lt;&gt;"VIGENTE")))</f>
-        <v/>
       </c>
       <c r="H15" t="n">
         <v>4</v>
@@ -15932,23 +15899,18 @@
       </c>
       <c r="B16" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H16,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$BF$2:$BF$1000)</f>
-        <v/>
       </c>
       <c r="C16" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H16,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CA$2:$CA$1000)</f>
-        <v/>
       </c>
       <c r="D16" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H16,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CD$2:$CD$1000)</f>
-        <v/>
       </c>
       <c r="E16" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H16,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0))</f>
-        <v/>
       </c>
       <c r="F16" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H16,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*(--(fabi!$J$2:$J$1000&lt;&gt;"VIGENTE")))</f>
-        <v/>
       </c>
       <c r="H16" t="n">
         <v>5</v>
@@ -15962,23 +15924,18 @@
       </c>
       <c r="B17" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H17,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$BF$2:$BF$1000)</f>
-        <v/>
       </c>
       <c r="C17" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H17,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CA$2:$CA$1000)</f>
-        <v/>
       </c>
       <c r="D17" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H17,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CD$2:$CD$1000)</f>
-        <v/>
       </c>
       <c r="E17" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H17,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0))</f>
-        <v/>
       </c>
       <c r="F17" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H17,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*(--(fabi!$J$2:$J$1000&lt;&gt;"VIGENTE")))</f>
-        <v/>
       </c>
       <c r="H17" t="n">
         <v>6</v>
@@ -15992,23 +15949,18 @@
       </c>
       <c r="B18" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H18,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$BF$2:$BF$1000)</f>
-        <v/>
       </c>
       <c r="C18" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H18,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CA$2:$CA$1000)</f>
-        <v/>
       </c>
       <c r="D18" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H18,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CD$2:$CD$1000)</f>
-        <v/>
       </c>
       <c r="E18" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H18,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0))</f>
-        <v/>
       </c>
       <c r="F18" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H18,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*(--(fabi!$J$2:$J$1000&lt;&gt;"VIGENTE")))</f>
-        <v/>
       </c>
       <c r="H18" t="n">
         <v>7</v>
@@ -16022,23 +15974,18 @@
       </c>
       <c r="B19" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H19,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$BF$2:$BF$1000)</f>
-        <v/>
       </c>
       <c r="C19" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H19,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CA$2:$CA$1000)</f>
-        <v/>
       </c>
       <c r="D19" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H19,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CD$2:$CD$1000)</f>
-        <v/>
       </c>
       <c r="E19" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H19,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0))</f>
-        <v/>
       </c>
       <c r="F19" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H19,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*(--(fabi!$J$2:$J$1000&lt;&gt;"VIGENTE")))</f>
-        <v/>
       </c>
       <c r="H19" t="n">
         <v>8</v>
@@ -16052,23 +15999,18 @@
       </c>
       <c r="B20" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H20,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$BF$2:$BF$1000)</f>
-        <v/>
       </c>
       <c r="C20" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H20,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CA$2:$CA$1000)</f>
-        <v/>
       </c>
       <c r="D20" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H20,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CD$2:$CD$1000)</f>
-        <v/>
       </c>
       <c r="E20" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H20,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0))</f>
-        <v/>
       </c>
       <c r="F20" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H20,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*(--(fabi!$J$2:$J$1000&lt;&gt;"VIGENTE")))</f>
-        <v/>
       </c>
       <c r="H20" t="n">
         <v>9</v>
@@ -16082,23 +16024,18 @@
       </c>
       <c r="B21" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H21,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$BF$2:$BF$1000)</f>
-        <v/>
       </c>
       <c r="C21" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H21,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CA$2:$CA$1000)</f>
-        <v/>
       </c>
       <c r="D21" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H21,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CD$2:$CD$1000)</f>
-        <v/>
       </c>
       <c r="E21" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H21,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0))</f>
-        <v/>
       </c>
       <c r="F21" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H21,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*(--(fabi!$J$2:$J$1000&lt;&gt;"VIGENTE")))</f>
-        <v/>
       </c>
       <c r="H21" t="n">
         <v>10</v>
@@ -16112,23 +16049,18 @@
       </c>
       <c r="B22" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H22,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$BF$2:$BF$1000)</f>
-        <v/>
       </c>
       <c r="C22" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H22,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CA$2:$CA$1000)</f>
-        <v/>
       </c>
       <c r="D22" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H22,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CD$2:$CD$1000)</f>
-        <v/>
       </c>
       <c r="E22" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H22,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0))</f>
-        <v/>
       </c>
       <c r="F22" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H22,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*(--(fabi!$J$2:$J$1000&lt;&gt;"VIGENTE")))</f>
-        <v/>
       </c>
       <c r="H22" t="n">
         <v>11</v>
@@ -16142,23 +16074,18 @@
       </c>
       <c r="B23" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H23,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$BF$2:$BF$1000)</f>
-        <v/>
       </c>
       <c r="C23" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H23,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CA$2:$CA$1000)</f>
-        <v/>
       </c>
       <c r="D23" s="10">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H23,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*fabi!$CD$2:$CD$1000)</f>
-        <v/>
       </c>
       <c r="E23" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H23,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0))</f>
-        <v/>
       </c>
       <c r="F23" s="11">
         <f>SUMPRODUCT((--(fabi!$R$2:$R$1000&amp;""=TEXT($H23,"00")))*((($C$4="")+(fabi!$F$2:$F$1000=$C$4))&gt;0)*(--(fabi!$J$2:$J$1000&lt;&gt;"VIGENTE")))</f>
-        <v/>
       </c>
       <c r="H23" t="n">
         <v>12</v>
@@ -16172,23 +16099,18 @@
       </c>
       <c r="B24" s="13">
         <f>SUM(B12:B23)</f>
-        <v/>
       </c>
       <c r="C24" s="13">
         <f>SUM(C12:C23)</f>
-        <v/>
       </c>
       <c r="D24" s="13">
         <f>SUM(D12:D23)</f>
-        <v/>
       </c>
       <c r="E24" s="14">
         <f>SUM(E12:E23)</f>
-        <v/>
       </c>
       <c r="F24" s="14">
         <f>SUM(F12:F23)</f>
-        <v/>
       </c>
     </row>
   </sheetData>
@@ -16197,7 +16119,7 @@
       <formula1>"1,2,3,4,5,6,7,8,9,10,11,12"</formula1>
     </dataValidation>
     <dataValidation sqref="C4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>fabi!$F$2:$F$1000</formula1>
+      <formula1>RFCList</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix definitivo tabla Gastos (table3.xml con estructura completa Excel) + ruta PQ real
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016pudwoamudm6kkBbcBjEzD
</commit_message>
<xml_diff>
--- a/Concentrado_CFDI_AUTOMATIZADO.xlsx
+++ b/Concentrado_CFDI_AUTOMATIZADO.xlsx
@@ -7793,16 +7793,16 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Gastos" displayName="Gastos" ref="A4:E28" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0000000B-000C-0000-FFFF-FFFF0B000000}" name="Gastos" displayName="Gastos" ref="A4:E28" totalsRowShown="0" headerRowCount="1">
   <autoFilter ref="A4:E28"/>
   <tableColumns count="5">
-    <tableColumn id="1" name="Mes"/>
-    <tableColumn id="2" name="Categoria"/>
-    <tableColumn id="3" name="Concepto"/>
-    <tableColumn id="4" name="Importe"/>
-    <tableColumn id="5" name="Origen"/>
+    <tableColumn id="1" xr3:uid="{0000000B-0010-0000-FFFF-FFFF01000000}" name="Mes"/>
+    <tableColumn id="2" xr3:uid="{0000000B-0010-0000-FFFF-FFFF02000000}" name="Categoria"/>
+    <tableColumn id="3" xr3:uid="{0000000B-0010-0000-FFFF-FFFF03000000}" name="Concepto"/>
+    <tableColumn id="4" xr3:uid="{0000000B-0010-0000-FFFF-FFFF04000000}" name="Importe"/>
+    <tableColumn id="5" xr3:uid="{0000000B-0010-0000-FFFF-FFFF05000000}" name="Origen"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 

</xml_diff>

<commit_message>
Fix definitivo: 'Gastos captura' sin ListObject (rango fijo + SUMIFS) para eliminar el aviso de reparación de Excel
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016pudwoamudm6kkBbcBjEzD
</commit_message>
<xml_diff>
--- a/Concentrado_CFDI_AUTOMATIZADO.xlsx
+++ b/Concentrado_CFDI_AUTOMATIZADO.xlsx
@@ -7792,20 +7792,6 @@
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0000000B-000C-0000-FFFF-FFFF0B000000}" name="Gastos" displayName="Gastos" ref="A4:E28" totalsRowShown="0" headerRowCount="1">
-  <autoFilter ref="A4:E28"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{0000000B-0010-0000-FFFF-FFFF01000000}" name="Mes"/>
-    <tableColumn id="2" xr3:uid="{0000000B-0010-0000-FFFF-FFFF02000000}" name="Categoria"/>
-    <tableColumn id="3" xr3:uid="{0000000B-0010-0000-FFFF-FFFF03000000}" name="Concepto"/>
-    <tableColumn id="4" xr3:uid="{0000000B-0010-0000-FFFF-FFFF04000000}" name="Importe"/>
-    <tableColumn id="5" xr3:uid="{0000000B-0010-0000-FFFF-FFFF05000000}" name="Origen"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
@@ -9421,7 +9407,7 @@
         </is>
       </c>
       <c r="I6" s="9">
-        <f>SUMIFS(Gastos[Importe],Gastos[Categoria],"Basico",Gastos[Mes],$I$3)</f>
+        <f>SUMIFS($D$5:$D$504,$B$5:$B$504,"Basico",$A$5:$A$504,$I$3)</f>
       </c>
       <c r="J6" s="10">
         <f>IFERROR(I6/$I$9,0)</f>
@@ -9455,7 +9441,7 @@
         </is>
       </c>
       <c r="I7" s="9">
-        <f>SUMIFS(Gastos[Importe],Gastos[Categoria],"Lujo",Gastos[Mes],$I$3)</f>
+        <f>SUMIFS($D$5:$D$504,$B$5:$B$504,"Lujo",$A$5:$A$504,$I$3)</f>
       </c>
       <c r="J7" s="10">
         <f>IFERROR(I7/$I$9,0)</f>
@@ -9489,7 +9475,7 @@
         </is>
       </c>
       <c r="I8" s="9">
-        <f>SUMIFS(Gastos[Importe],Gastos[Categoria],"Ahorro",Gastos[Mes],$I$3)</f>
+        <f>SUMIFS($D$5:$D$504,$B$5:$B$504,"Ahorro",$A$5:$A$504,$I$3)</f>
       </c>
       <c r="J8" s="10">
         <f>IFERROR(I8/$I$9,0)</f>
@@ -9908,13 +9894,13 @@
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation sqref="B5:B28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B5:B504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Basico,Lujo,Ahorro"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E5:E504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Manual,XML"</formula1>
     </dataValidation>
-    <dataValidation sqref="A5:A28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A5:A504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"1,2,3,4,5,6,7,8,9,10,11,12"</formula1>
     </dataValidation>
     <dataValidation sqref="I3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -9923,9 +9909,6 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>